<commit_message>
Remove legacy card table assets
</commit_message>
<xml_diff>
--- a/project-a/tables/ProjectDataTables.xlsx
+++ b/project-a/tables/ProjectDataTables.xlsx
@@ -2,16 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5def65f1ca614480"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cards" sheetId="2" r:id="R37a8f6b1cb0346fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="character_cards" sheetId="3" r:id="R4c54615ba6b14954"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="card_effects" sheetId="4" r:id="Re8353ba02a4f427e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="player_growth" sheetId="5" r:id="Rdb7166620c224b47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="player_stats_current" sheetId="6" r:id="Rb58df6e1c8504bf9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="monster_stats" sheetId="7" r:id="R0cf0e6988fbe4606"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="monsters" sheetId="8" r:id="Re1ebd8fe697a41cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="monster_intents" sheetId="9" r:id="R329d132925c74f1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SourceAudit" sheetId="10" r:id="Rdb0daf56129e461b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rad09b49f7ba34e09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="character_cards" sheetId="2" r:id="R1c80304bdc754e88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="card_effects" sheetId="3" r:id="R40bade777bd94c7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="player_growth" sheetId="4" r:id="R36f706580ff6408a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="player_stats_current" sheetId="5" r:id="R33cd7580307a40f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="monster_stats" sheetId="6" r:id="R8521993afd5847dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="monsters" sheetId="7" r:id="R0a4d1ed6dae34b8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="monster_intents" sheetId="8" r:id="R129cedb5d46a4a76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SourceAudit" sheetId="9" r:id="R357027218ab84a26"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -105,7 +104,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="22">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -131,13 +130,6 @@
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <x:extLst>
-        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
-        </x:ext>
-      </x:extLst>
-    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -147,64 +139,17 @@
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <x:extLst>
-        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
-        </x:ext>
-      </x:extLst>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <x:extLst>
-        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
-        </x:ext>
-      </x:extLst>
-    </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-      <x:extLst>
-        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
-        </x:ext>
-      </x:extLst>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-      <x:extLst>
-        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
-        </x:ext>
-      </x:extLst>
-    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
-</file>
-
-<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
-<xfpb:FeaturePropertyBags xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
-  <xfpb:bag type="Checkbox"/>
-  <xfpb:bag type="XFControls">
-    <xfpb:bagId k="CellControl">0</xfpb:bagId>
-  </xfpb:bag>
-  <xfpb:bag type="XFComplement">
-    <xfpb:bagId k="XFControls">1</xfpb:bagId>
-  </xfpb:bag>
-  <xfpb:bag type="XFComplements" extRef="XFComplementsMapperExtRef">
-    <xfpb:a k="MappedFeaturePropertyBags">
-      <xfpb:bagId>2</xfpb:bagId>
-    </xfpb:a>
-  </xfpb:bag>
-</xfpb:FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -464,121 +409,115 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="5" t="str">
-        <x:v>Base cards</x:v>
+        <x:v>Tsuki character cards</x:v>
       </x:c>
       <x:c r="B5" s="5" t="n">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C5" s="5" t="str">
-        <x:v>Legacy/fallback cards</x:v>
+        <x:v>Active deck data</x:v>
       </x:c>
       <x:c r="D5" s="5" t="str">
-        <x:v>tables/excel/CardTable.xlsx</x:v>
+        <x:v>tables/excel/CharacterCards.xlsx</x:v>
       </x:c>
       <x:c r="E5" s="5" t="str">
-        <x:v>Decide whether to keep after Tsuki deck migration</x:v>
-      </x:c>
-      <x:c r="F5" s="5" t="str"/>
-    </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
+        <x:v>Keep Korean text in Excel as source of truth</x:v>
+      </x:c>
+      <x:c r="F5" s="5" t="str">
+        <x:v>Legacy CardTable/cards.json retired</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A6" s="5" t="str">
-        <x:v>Tsuki character cards</x:v>
+        <x:v>Player growth</x:v>
       </x:c>
       <x:c r="B6" s="5" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C6" s="5" t="str">
+        <x:v>Authoring/reference</x:v>
+      </x:c>
+      <x:c r="D6" s="5" t="str">
+        <x:v>tables/excel/StatTable.xlsx</x:v>
+      </x:c>
+      <x:c r="E6" s="5" t="str">
+        <x:v>Connect to character progression when screen exists</x:v>
+      </x:c>
+      <x:c r="F6" s="5"/>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="5" t="str">
+        <x:v>Monster stats</x:v>
+      </x:c>
+      <x:c r="B7" s="5" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="C6" s="5" t="str">
-        <x:v>Active deck data</x:v>
-      </x:c>
-      <x:c r="D6" s="5" t="str">
-        <x:v>tables/excel/CharacterCards.xlsx</x:v>
-      </x:c>
-      <x:c r="E6" s="5" t="str">
-        <x:v>Keep Korean text in Excel as source of truth</x:v>
-      </x:c>
-      <x:c r="F6" s="5" t="str"/>
-    </x:row>
-    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A7" s="5" t="str">
-        <x:v>Player growth</x:v>
-      </x:c>
-      <x:c r="B7" s="5" t="n">
+      <x:c r="C7" s="5" t="str">
+        <x:v>Stats .tres mirror</x:v>
+      </x:c>
+      <x:c r="D7" s="5" t="str">
+        <x:v>data/monsters/*Stats.tres</x:v>
+      </x:c>
+      <x:c r="E7" s="5" t="str">
+        <x:v>Use this sheet for balance review</x:v>
+      </x:c>
+      <x:c r="F7" s="5"/>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="5" t="str">
+        <x:v>Monster metadata</x:v>
+      </x:c>
+      <x:c r="B8" s="5" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="C7" s="5" t="str">
-        <x:v>Authoring/reference</x:v>
-      </x:c>
-      <x:c r="D7" s="5" t="str">
-        <x:v>tables/excel/StatTable.xlsx</x:v>
-      </x:c>
-      <x:c r="E7" s="5" t="str">
-        <x:v>Connect to character progression when screen exists</x:v>
-      </x:c>
-      <x:c r="F7" s="5" t="str"/>
-    </x:row>
-    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A8" s="5" t="str">
-        <x:v>Monster stats</x:v>
-      </x:c>
-      <x:c r="B8" s="5" t="n">
-        <x:v>8</x:v>
-      </x:c>
       <x:c r="C8" s="5" t="str">
-        <x:v>Stats .tres mirror</x:v>
+        <x:v>Active combat data</x:v>
       </x:c>
       <x:c r="D8" s="5" t="str">
-        <x:v>data/monsters/*Stats.tres</x:v>
+        <x:v>data/monsters/*.tres</x:v>
       </x:c>
       <x:c r="E8" s="5" t="str">
-        <x:v>Use this sheet for balance review</x:v>
+        <x:v>Consider exporter/importer support later</x:v>
       </x:c>
       <x:c r="F8" s="5" t="str">
-        <x:v>Existing StatTable.xlsx updated with all current monsters</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
+        <x:v>Scene, intents, action count, UI offsets</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A9" s="5" t="str">
-        <x:v>Monster metadata</x:v>
+        <x:v>Monster intents</x:v>
       </x:c>
       <x:c r="B9" s="5" t="n">
-        <x:v>7</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C9" s="5" t="str">
         <x:v>Active combat data</x:v>
       </x:c>
       <x:c r="D9" s="5" t="str">
-        <x:v>data/monsters/*.tres</x:v>
+        <x:v>data/monsters/intents/*.tres</x:v>
       </x:c>
       <x:c r="E9" s="5" t="str">
-        <x:v>Consider exporter/importer support later</x:v>
-      </x:c>
-      <x:c r="F9" s="5" t="str">
-        <x:v>Scene, intents, action count, UI offsets</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A10" s="5" t="str">
-        <x:v>Monster intents</x:v>
-      </x:c>
-      <x:c r="B10" s="5" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C10" s="5" t="str">
-        <x:v>Active combat data</x:v>
-      </x:c>
-      <x:c r="D10" s="5" t="str">
-        <x:v>data/monsters/intents/*.tres</x:v>
-      </x:c>
-      <x:c r="E10" s="5" t="str">
         <x:v>Expand intent table as new behavior types appear</x:v>
       </x:c>
-      <x:c r="F10" s="5" t="str"/>
+      <x:c r="F9" s="5"/>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="5"/>
+      <x:c r="B10" s="5"/>
+      <x:c r="C10" s="5"/>
+      <x:c r="D10" s="5"/>
+      <x:c r="E10" s="5"/>
+      <x:c r="F10" s="5"/>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="5"/>
-      <x:c r="B11" s="5"/>
+      <x:c r="A11" s="5" t="str">
+        <x:v>Player snapshot</x:v>
+      </x:c>
+      <x:c r="B11" s="5" t="str">
+        <x:v>Value</x:v>
+      </x:c>
       <x:c r="C11" s="5"/>
       <x:c r="D11" s="5"/>
       <x:c r="E11" s="5"/>
@@ -586,10 +525,10 @@
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="5" t="str">
-        <x:v>Player snapshot</x:v>
-      </x:c>
-      <x:c r="B12" s="5" t="str">
-        <x:v>Value</x:v>
+        <x:v>max_hp</x:v>
+      </x:c>
+      <x:c r="B12" s="5" t="n">
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C12" s="5"/>
       <x:c r="D12" s="5"/>
@@ -598,10 +537,10 @@
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="5" t="str">
-        <x:v>max_hp</x:v>
+        <x:v>attack_power</x:v>
       </x:c>
       <x:c r="B13" s="5" t="n">
-        <x:v>90</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="C13" s="5"/>
       <x:c r="D13" s="5"/>
@@ -610,10 +549,10 @@
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="5" t="str">
-        <x:v>attack_power</x:v>
+        <x:v>defense_power</x:v>
       </x:c>
       <x:c r="B14" s="5" t="n">
-        <x:v>160</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C14" s="5"/>
       <x:c r="D14" s="5"/>
@@ -621,28 +560,16 @@
       <x:c r="F14" s="5"/>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
-      <x:c r="A15" s="5" t="str">
-        <x:v>defense_power</x:v>
-      </x:c>
-      <x:c r="B15" s="5" t="n">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="C15" s="5"/>
-      <x:c r="D15" s="5"/>
-      <x:c r="E15" s="5"/>
-      <x:c r="F15" s="5"/>
-    </x:row>
-    <x:row r="16" ht="15" hidden="0" customHeight="1">
-      <x:c r="A16" s="6" t="str">
+      <x:c r="A15" s="6" t="str">
         <x:v>starting_energy</x:v>
       </x:c>
-      <x:c r="B16" s="6" t="n">
+      <x:c r="B15" s="6" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C16" s="6"/>
-      <x:c r="D16" s="6"/>
-      <x:c r="E16" s="6"/>
-      <x:c r="F16" s="6"/>
+      <x:c r="C15" s="6"/>
+      <x:c r="D15" s="6"/>
+      <x:c r="E15" s="6"/>
+      <x:c r="F15" s="6"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -652,290 +579,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="90" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="4" t="str">
-        <x:v>Item</x:v>
-      </x:c>
-      <x:c r="B1" s="4" t="str">
-        <x:v>Status</x:v>
-      </x:c>
-      <x:c r="C1" s="4" t="str">
-        <x:v>Detail</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="5" t="str">
-        <x:v>CardTable.xlsx</x:v>
-      </x:c>
-      <x:c r="B2" s="5" t="str">
-        <x:v>kept</x:v>
-      </x:c>
-      <x:c r="C2" s="5" t="str">
-        <x:v>Legacy/fallback card sheet remains exporter-compatible.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="5" t="str">
-        <x:v>CharacterCards.xlsx</x:v>
-      </x:c>
-      <x:c r="B3" s="5" t="str">
-        <x:v>kept</x:v>
-      </x:c>
-      <x:c r="C3" s="5" t="str">
-        <x:v>Active Tsuki card sheet and glossary remain exporter-compatible.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="5" t="str">
-        <x:v>StatTable.xlsx</x:v>
-      </x:c>
-      <x:c r="B4" s="5" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="C4" s="5" t="str">
-        <x:v>monster_stats now includes current monster Stats.tres files.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="5" t="str">
-        <x:v>ProjectDataTables.xlsx</x:v>
-      </x:c>
-      <x:c r="B5" s="5" t="str">
-        <x:v>new</x:v>
-      </x:c>
-      <x:c r="C5" s="5" t="str">
-        <x:v>Integrated balancing/reference workbook outside tables/excel to avoid duplicate exporter output.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="6" t="str">
-        <x:v>Monster .tres files</x:v>
-      </x:c>
-      <x:c r="B6" s="6" t="str">
-        <x:v>source</x:v>
-      </x:c>
-      <x:c r="C6" s="6" t="str">
-        <x:v>Runtime preloads these directly in scripts/core/ingame.gd.</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="58" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A1" s="4" t="str">
-        <x:v>TABLE SCRIPT</x:v>
-      </x:c>
-      <x:c r="B1" s="4" t="str">
-        <x:v>Generated/organized by Codex. Row 2 is #data for exporter-compatible sheets.</x:v>
-      </x:c>
-      <x:c r="C1" s="4"/>
-      <x:c r="D1" s="4"/>
-      <x:c r="E1" s="4"/>
-      <x:c r="F1" s="4"/>
-      <x:c r="G1" s="4"/>
-      <x:c r="H1" s="4"/>
-    </x:row>
-    <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="10" t="str">
-        <x:v>#data</x:v>
-      </x:c>
-      <x:c r="B2" s="10" t="str">
-        <x:v>id</x:v>
-      </x:c>
-      <x:c r="C2" s="10" t="str">
-        <x:v>display_name</x:v>
-      </x:c>
-      <x:c r="D2" s="10" t="str">
-        <x:v>cost</x:v>
-      </x:c>
-      <x:c r="E2" s="10" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="F2" s="10" t="str">
-        <x:v>card_type</x:v>
-      </x:c>
-      <x:c r="G2" s="10" t="str">
-        <x:v>requires_target</x:v>
-      </x:c>
-      <x:c r="H2" s="10" t="str">
-        <x:v>effects</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="23"/>
-      <x:c r="B3" s="23" t="str">
-        <x:v>key,string</x:v>
-      </x:c>
-      <x:c r="C3" s="23" t="str">
-        <x:v>string</x:v>
-      </x:c>
-      <x:c r="D3" s="23" t="str">
-        <x:v>int</x:v>
-      </x:c>
-      <x:c r="E3" s="23" t="str">
-        <x:v>string</x:v>
-      </x:c>
-      <x:c r="F3" s="23" t="str">
-        <x:v>string</x:v>
-      </x:c>
-      <x:c r="G3" s="23" t="str">
-        <x:v>bool</x:v>
-      </x:c>
-      <x:c r="H3" s="23" t="str">
-        <x:v>json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="24"/>
-      <x:c r="B4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="C4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="D4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="E4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="F4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="G4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="H4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="5"/>
-      <x:c r="B5" s="5" t="str">
-        <x:v>slash</x:v>
-      </x:c>
-      <x:c r="C5" s="5" t="str">
-        <x:v>베기</x:v>
-      </x:c>
-      <x:c r="D5" s="5" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E5" s="5" t="str">
-        <x:v>피해 6을 줍니다.</x:v>
-      </x:c>
-      <x:c r="F5" s="5" t="str">
-        <x:v>attack</x:v>
-      </x:c>
-      <x:c r="G5" s="25" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H5" s="5" t="str">
-        <x:v>[{"type": "damage", "amount": 6, "target": "enemy"}]</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="5"/>
-      <x:c r="B6" s="5" t="str">
-        <x:v>guard</x:v>
-      </x:c>
-      <x:c r="C6" s="5" t="str">
-        <x:v>방어</x:v>
-      </x:c>
-      <x:c r="D6" s="5" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E6" s="5" t="str">
-        <x:v>방어도 7을 얻습니다.</x:v>
-      </x:c>
-      <x:c r="F6" s="5" t="str">
-        <x:v>skill</x:v>
-      </x:c>
-      <x:c r="G6" s="25" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H6" s="5" t="str">
-        <x:v>[{"type": "block", "amount": 7, "target": "self"}]</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="5"/>
-      <x:c r="B7" s="5" t="str">
-        <x:v>focus</x:v>
-      </x:c>
-      <x:c r="C7" s="5" t="str">
-        <x:v>집중</x:v>
-      </x:c>
-      <x:c r="D7" s="5" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E7" s="5" t="str">
-        <x:v>카드 1장을 뽑고 에너지 1을 얻습니다.</x:v>
-      </x:c>
-      <x:c r="F7" s="5" t="str">
-        <x:v>skill</x:v>
-      </x:c>
-      <x:c r="G7" s="25" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H7" s="5" t="str">
-        <x:v>[{"type": "draw", "amount": 1}, {"type": "energy", "amount": 1}]</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="6"/>
-      <x:c r="B8" s="6" t="str">
-        <x:v>heavy_slash</x:v>
-      </x:c>
-      <x:c r="C8" s="6" t="str">
-        <x:v>강타</x:v>
-      </x:c>
-      <x:c r="D8" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E8" s="6" t="str">
-        <x:v>피해 12를 줍니다.</x:v>
-      </x:c>
-      <x:c r="F8" s="6" t="str">
-        <x:v>attack</x:v>
-      </x:c>
-      <x:c r="G8" s="26" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H8" s="6" t="str">
-        <x:v>[{"type": "damage", "amount": 12, "target": "enemy"}]</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1005,68 +649,68 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="23"/>
-      <x:c r="B3" s="23" t="str">
+      <x:c r="A3" s="20"/>
+      <x:c r="B3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
-      <x:c r="C3" s="23" t="str">
+      <x:c r="C3" s="20" t="str">
         <x:v>key,string</x:v>
       </x:c>
-      <x:c r="D3" s="23" t="str">
+      <x:c r="D3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
-      <x:c r="E3" s="23" t="str">
+      <x:c r="E3" s="20" t="str">
         <x:v>int</x:v>
       </x:c>
-      <x:c r="F3" s="23" t="str">
+      <x:c r="F3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
-      <x:c r="G3" s="23" t="str">
+      <x:c r="G3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
-      <x:c r="H3" s="23" t="str">
+      <x:c r="H3" s="20" t="str">
         <x:v>int</x:v>
       </x:c>
-      <x:c r="I3" s="23" t="str">
+      <x:c r="I3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
-      <x:c r="J3" s="23" t="str">
+      <x:c r="J3" s="20" t="str">
         <x:v>json</x:v>
       </x:c>
-      <x:c r="K3" s="23" t="str">
+      <x:c r="K3" s="20" t="str">
         <x:v>json,null</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="24"/>
-      <x:c r="B4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="C4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="D4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="E4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="F4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="G4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="H4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="I4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="J4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="K4" s="24" t="str">
+      <x:c r="A4" s="21"/>
+      <x:c r="B4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="C4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="D4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="E4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="F4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="G4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="H4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="I4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="J4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="K4" s="21" t="str">
         <x:v>data</x:v>
       </x:c>
     </x:row>
@@ -1319,7 +963,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1354,26 +998,26 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="23"/>
-      <x:c r="B3" s="23" t="str">
+      <x:c r="A3" s="20"/>
+      <x:c r="B3" s="20" t="str">
         <x:v>key,string</x:v>
       </x:c>
-      <x:c r="C3" s="23" t="str">
+      <x:c r="C3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
-      <x:c r="D3" s="23" t="str">
+      <x:c r="D3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="24"/>
-      <x:c r="B4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="C4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="D4" s="24" t="str">
+      <x:c r="A4" s="21"/>
+      <x:c r="B4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="C4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="D4" s="21" t="str">
         <x:v>data</x:v>
       </x:c>
     </x:row>
@@ -1994,7 +1638,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2049,50 +1693,50 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="23"/>
-      <x:c r="B3" s="23" t="str">
+      <x:c r="A3" s="20"/>
+      <x:c r="B3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
-      <x:c r="C3" s="23" t="str">
+      <x:c r="C3" s="20" t="str">
         <x:v>key,int</x:v>
       </x:c>
-      <x:c r="D3" s="23" t="str">
+      <x:c r="D3" s="20" t="str">
         <x:v>int</x:v>
       </x:c>
-      <x:c r="E3" s="23" t="str">
+      <x:c r="E3" s="20" t="str">
         <x:v>int</x:v>
       </x:c>
-      <x:c r="F3" s="23" t="str">
+      <x:c r="F3" s="20" t="str">
         <x:v>int</x:v>
       </x:c>
-      <x:c r="G3" s="23" t="str">
+      <x:c r="G3" s="20" t="str">
         <x:v>float</x:v>
       </x:c>
-      <x:c r="H3" s="23" t="str">
+      <x:c r="H3" s="20" t="str">
         <x:v>float</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="24"/>
-      <x:c r="B4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="C4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="D4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="E4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="F4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="G4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="H4" s="24" t="str">
+      <x:c r="A4" s="21"/>
+      <x:c r="B4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="C4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="D4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="E4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="F4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="G4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="H4" s="21" t="str">
         <x:v>data</x:v>
       </x:c>
     </x:row>
@@ -2269,7 +1913,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2362,7 +2006,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2422,56 +2066,56 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="23"/>
-      <x:c r="B3" s="23" t="str">
+      <x:c r="A3" s="20"/>
+      <x:c r="B3" s="20" t="str">
         <x:v>key,string</x:v>
       </x:c>
-      <x:c r="C3" s="23" t="str">
+      <x:c r="C3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
-      <x:c r="D3" s="23" t="str">
+      <x:c r="D3" s="20" t="str">
         <x:v>int</x:v>
       </x:c>
-      <x:c r="E3" s="23" t="str">
+      <x:c r="E3" s="20" t="str">
         <x:v>int</x:v>
       </x:c>
-      <x:c r="F3" s="23" t="str">
+      <x:c r="F3" s="20" t="str">
         <x:v>int</x:v>
       </x:c>
-      <x:c r="G3" s="23" t="str">
+      <x:c r="G3" s="20" t="str">
         <x:v>float</x:v>
       </x:c>
-      <x:c r="H3" s="23" t="str">
+      <x:c r="H3" s="20" t="str">
         <x:v>float</x:v>
       </x:c>
-      <x:c r="I3" s="23" t="str">
+      <x:c r="I3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="24"/>
-      <x:c r="B4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="C4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="D4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="E4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="F4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="G4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="H4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="I4" s="24" t="str">
+      <x:c r="A4" s="21"/>
+      <x:c r="B4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="C4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="D4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="E4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="F4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="G4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="H4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="I4" s="21" t="str">
         <x:v>data</x:v>
       </x:c>
     </x:row>
@@ -2696,7 +2340,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2761,62 +2405,62 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="23"/>
-      <x:c r="B3" s="23" t="str">
+      <x:c r="A3" s="20"/>
+      <x:c r="B3" s="20" t="str">
         <x:v>key,string</x:v>
       </x:c>
-      <x:c r="C3" s="23" t="str">
+      <x:c r="C3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
-      <x:c r="D3" s="23" t="str">
+      <x:c r="D3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
-      <x:c r="E3" s="23" t="str">
+      <x:c r="E3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
-      <x:c r="F3" s="23" t="str">
+      <x:c r="F3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
-      <x:c r="G3" s="23" t="str">
+      <x:c r="G3" s="20" t="str">
         <x:v>int</x:v>
       </x:c>
-      <x:c r="H3" s="23" t="str">
+      <x:c r="H3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
-      <x:c r="I3" s="23" t="str">
+      <x:c r="I3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
-      <x:c r="J3" s="23" t="str">
+      <x:c r="J3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="24"/>
-      <x:c r="B4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="C4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="D4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="E4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="F4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="G4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="H4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="I4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="J4" s="24" t="str">
+      <x:c r="A4" s="21"/>
+      <x:c r="B4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="C4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="D4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="E4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="F4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="G4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="H4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="I4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="J4" s="21" t="str">
         <x:v>data</x:v>
       </x:c>
     </x:row>
@@ -3035,7 +2679,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -3090,50 +2734,50 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="23"/>
-      <x:c r="B3" s="23" t="str">
+      <x:c r="A3" s="20"/>
+      <x:c r="B3" s="20" t="str">
         <x:v>key,string</x:v>
       </x:c>
-      <x:c r="C3" s="23" t="str">
+      <x:c r="C3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
-      <x:c r="D3" s="23" t="str">
+      <x:c r="D3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
-      <x:c r="E3" s="23" t="str">
+      <x:c r="E3" s="20" t="str">
         <x:v>int</x:v>
       </x:c>
-      <x:c r="F3" s="23" t="str">
+      <x:c r="F3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
-      <x:c r="G3" s="23" t="str">
+      <x:c r="G3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
-      <x:c r="H3" s="23" t="str">
+      <x:c r="H3" s="20" t="str">
         <x:v>string</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="24"/>
-      <x:c r="B4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="C4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="D4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="E4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="F4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="G4" s="24" t="str">
-        <x:v>data</x:v>
-      </x:c>
-      <x:c r="H4" s="24" t="str">
+      <x:c r="A4" s="21"/>
+      <x:c r="B4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="C4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="D4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="E4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="F4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="G4" s="21" t="str">
+        <x:v>data</x:v>
+      </x:c>
+      <x:c r="H4" s="21" t="str">
         <x:v>data</x:v>
       </x:c>
     </x:row>
@@ -3212,4 +2856,84 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="42" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="90" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Item</x:v>
+      </x:c>
+      <x:c r="B1" s="4" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="C1" s="4" t="str">
+        <x:v>Detail</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="5" t="str">
+        <x:v>CharacterCards.xlsx</x:v>
+      </x:c>
+      <x:c r="B2" s="5" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="C2" s="5" t="str">
+        <x:v>Active Tsuki card sheet and glossary remain exporter-compatible.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="5" t="str">
+        <x:v>StatTable.xlsx</x:v>
+      </x:c>
+      <x:c r="B3" s="5" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="C3" s="5" t="str">
+        <x:v>player_growth and monster_stats exporter-compatible sheets.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="5" t="str">
+        <x:v>ProjectDataTables.xlsx</x:v>
+      </x:c>
+      <x:c r="B4" s="5" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="C4" s="5" t="str">
+        <x:v>Integrated balancing/reference workbook outside tables/excel to avoid duplicate exporter output.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="5" t="str">
+        <x:v>CardTable.xlsx / cards.json / data/cards/*.tres</x:v>
+      </x:c>
+      <x:c r="B5" s="5" t="str">
+        <x:v>retired</x:v>
+      </x:c>
+      <x:c r="C5" s="5" t="str">
+        <x:v>No runtime or exporter dependency remains after cleanup.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>Monster .tres files</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="str">
+        <x:v>source</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="str">
+        <x:v>Runtime preloads these directly in scripts/core/ingame.gd.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Pascalize Excel source tables
</commit_message>
<xml_diff>
--- a/project-a/tables/ProjectDataTables.xlsx
+++ b/project-a/tables/ProjectDataTables.xlsx
@@ -4,15 +4,15 @@
   <workbookPr/>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="character_cards" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="card_effects" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="player_growth" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="player_stats_current" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="monster_stats" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="monsters" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="monster_intents" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CharacterCards" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CardEffects" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerGrowth" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsCurrent" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterStats" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monsters" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterIntents" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SourceAudit" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="card_effect_rows" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CardEffectRows" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -459,7 +459,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>Cards: generated/character_cards.json, Monsters: .tres preload</t>
+          <t>Cards: generated/CharacterCards.json, Monsters: .tres preload</t>
         </is>
       </c>
       <c r="F2" s="5" t="n"/>
@@ -669,7 +669,7 @@
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>max_hp</t>
+          <t>MaxHp</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
@@ -683,7 +683,7 @@
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>attack_power</t>
+          <t>Attack</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
@@ -697,7 +697,7 @@
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>defense_power</t>
+          <t>Defense</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
@@ -711,7 +711,7 @@
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>starting_energy</t>
+          <t>StartingEnergy</t>
         </is>
       </c>
       <c r="B15" s="6" t="n">
@@ -777,82 +777,82 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>Id</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>card_key</t>
+          <t>CardKey</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>character</t>
+          <t>Character</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>card_id</t>
+          <t>CardId</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>trigger</t>
+          <t>Trigger</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>stance</t>
+          <t>Stance</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>effect_type</t>
+          <t>EffectType</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>target</t>
+          <t>Target</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>card_type</t>
+          <t>CardType</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>buff</t>
+          <t>Buff</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>Percent</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>Amount</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>duration_turns</t>
+          <t>DurationTurns</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>scope</t>
+          <t>Scope</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>condition</t>
+          <t>Condition</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>text_arg_index</t>
+          <t>TextArgIndex</t>
         </is>
       </c>
     </row>
@@ -1023,37 +1023,37 @@
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>tsuki_crescent_slash_damage</t>
+          <t>TsukiCrescentSlashDamage</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>tsuki/crescent_slash</t>
+          <t>Tsuki/CrescentSlash</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>crescent_slash</t>
+          <t>CrescentSlash</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>on_play</t>
+          <t>OnPlay</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>Damage</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>enemy</t>
+          <t>Enemy</t>
         </is>
       </c>
       <c r="L5" t="n">
@@ -1066,27 +1066,27 @@
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>tsuki_crescent_slash_moon_shield</t>
+          <t>TsukiCrescentSlashMoonShield</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>tsuki/crescent_slash</t>
+          <t>Tsuki/CrescentSlash</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>crescent_slash</t>
+          <t>CrescentSlash</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>on_stance</t>
+          <t>OnStance</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1096,12 +1096,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>shield</t>
+          <t>Shield</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>Self</t>
         </is>
       </c>
       <c r="L6" t="n">
@@ -1114,27 +1114,27 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>tsuki_crescent_slash_sun_damage_up</t>
+          <t>TsukiCrescentSlashSunDamageUp</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>tsuki/crescent_slash</t>
+          <t>Tsuki/CrescentSlash</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>crescent_slash</t>
+          <t>CrescentSlash</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>on_stance</t>
+          <t>OnStance</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>damage_delta</t>
+          <t>DamageDelta</t>
         </is>
       </c>
       <c r="L7" t="n">
@@ -1157,37 +1157,37 @@
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>tsuki_flow_guard_shield</t>
+          <t>TsukiFlowGuardShield</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>tsuki/flow_guard</t>
+          <t>Tsuki/FlowGuard</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>flow_guard</t>
+          <t>FlowGuard</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>on_play</t>
+          <t>OnPlay</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>shield</t>
+          <t>Shield</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>Self</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -1200,27 +1200,27 @@
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>tsuki_flow_guard_moon_draw</t>
+          <t>TsukiFlowGuardMoonDraw</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>tsuki/flow_guard</t>
+          <t>Tsuki/FlowGuard</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>flow_guard</t>
+          <t>FlowGuard</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>on_stance</t>
+          <t>OnStance</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>draw</t>
+          <t>Draw</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -1243,27 +1243,27 @@
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
-          <t>tsuki_flow_guard_sun_buff</t>
+          <t>TsukiFlowGuardSunBuff</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>tsuki/flow_guard</t>
+          <t>Tsuki/FlowGuard</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>flow_guard</t>
+          <t>FlowGuard</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>on_stance</t>
+          <t>OnStance</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1273,12 +1273,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>buff</t>
+          <t>Buff</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>attack_damage_up</t>
+          <t>AttackDamageUp</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -1291,59 +1291,59 @@
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
-          <t>tsuki_stance_shift_change</t>
+          <t>TsukiStanceShiftChange</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>tsuki/stance_shift</t>
+          <t>Tsuki/StanceShift</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>stance_shift</t>
+          <t>StanceShift</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>on_play</t>
+          <t>OnPlay</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>stance_change</t>
+          <t>StanceChange</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
-          <t>tsuki_stance_shift_moon_draw</t>
+          <t>TsukiStanceShiftMoonDraw</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>tsuki/stance_shift</t>
+          <t>Tsuki/StanceShift</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>stance_shift</t>
+          <t>StanceShift</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>on_stance</t>
+          <t>OnStance</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>draw</t>
+          <t>Draw</t>
         </is>
       </c>
       <c r="M12" t="n">
@@ -1366,27 +1366,27 @@
     <row r="13">
       <c r="B13" t="inlineStr">
         <is>
-          <t>tsuki_stance_shift_sun_buff</t>
+          <t>TsukiStanceShiftSunBuff</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>tsuki/stance_shift</t>
+          <t>Tsuki/StanceShift</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>stance_shift</t>
+          <t>StanceShift</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>on_stance</t>
+          <t>OnStance</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1396,12 +1396,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>buff</t>
+          <t>Buff</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>attack_damage_up</t>
+          <t>AttackDamageUp</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -1414,37 +1414,37 @@
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
-          <t>tsuki_afterimage_thrust_damage_1</t>
+          <t>TsukiAfterimageThrustDamage1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>tsuki/afterimage_thrust</t>
+          <t>Tsuki/AfterimageThrust</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>afterimage_thrust</t>
+          <t>AfterimageThrust</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>on_play</t>
+          <t>OnPlay</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>Damage</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>enemy</t>
+          <t>Enemy</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1457,37 +1457,37 @@
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>tsuki_afterimage_thrust_damage_2</t>
+          <t>TsukiAfterimageThrustDamage2</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>tsuki/afterimage_thrust</t>
+          <t>Tsuki/AfterimageThrust</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>afterimage_thrust</t>
+          <t>AfterimageThrust</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>on_play</t>
+          <t>OnPlay</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>Damage</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>enemy</t>
+          <t>Enemy</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1497,27 +1497,27 @@
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
-          <t>tsuki_afterimage_thrust_moon_add_stance</t>
+          <t>TsukiAfterimageThrustMoonAddStance</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>tsuki/afterimage_thrust</t>
+          <t>Tsuki/AfterimageThrust</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>afterimage_thrust</t>
+          <t>AfterimageThrust</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>on_stance</t>
+          <t>OnStance</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>add_card_to_hand</t>
+          <t>AddCardToHand</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>stance_shift</t>
+          <t>StanceShift</t>
         </is>
       </c>
       <c r="Q16" t="n">
@@ -1545,27 +1545,27 @@
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>tsuki_afterimage_thrust_sun_extra_damage</t>
+          <t>TsukiAfterimageThrustSunExtraDamage</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>tsuki/afterimage_thrust</t>
+          <t>Tsuki/AfterimageThrust</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>afterimage_thrust</t>
+          <t>AfterimageThrust</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>on_stance</t>
+          <t>OnStance</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1575,12 +1575,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>Damage</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>enemy</t>
+          <t>Enemy</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1596,32 +1596,32 @@
     <row r="18">
       <c r="B18" t="inlineStr">
         <is>
-          <t>tsuki_breath_reset_draw</t>
+          <t>TsukiBreathResetDraw</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>tsuki/breath_reset</t>
+          <t>Tsuki/BreathReset</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>breath_reset</t>
+          <t>BreathReset</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>on_play</t>
+          <t>OnPlay</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>draw</t>
+          <t>Draw</t>
         </is>
       </c>
       <c r="M18" t="n">
@@ -1634,27 +1634,27 @@
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
-          <t>tsuki_breath_reset_moon_shield</t>
+          <t>TsukiBreathResetMoonShield</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>tsuki/breath_reset</t>
+          <t>Tsuki/BreathReset</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>breath_reset</t>
+          <t>BreathReset</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>on_stance</t>
+          <t>OnStance</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1664,12 +1664,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>shield</t>
+          <t>Shield</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>Self</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -1682,27 +1682,27 @@
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
-          <t>tsuki_breath_reset_sun_energy</t>
+          <t>TsukiBreathResetSunEnergy</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>tsuki/breath_reset</t>
+          <t>Tsuki/BreathReset</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>breath_reset</t>
+          <t>BreathReset</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>on_stance</t>
+          <t>OnStance</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>energy</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="M20" t="n">
@@ -1725,37 +1725,37 @@
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
-          <t>tsuki_rupture_cleave_damage</t>
+          <t>TsukiRuptureCleaveDamage</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>tsuki/rupture_cleave</t>
+          <t>Tsuki/RuptureCleave</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>rupture_cleave</t>
+          <t>RuptureCleave</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>on_play</t>
+          <t>OnPlay</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>Damage</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>all_enemies</t>
+          <t>AllEnemies</t>
         </is>
       </c>
       <c r="L21" t="n">
@@ -1768,27 +1768,27 @@
     <row r="22">
       <c r="B22" t="inlineStr">
         <is>
-          <t>tsuki_rupture_cleave_moon_shield</t>
+          <t>TsukiRuptureCleaveMoonShield</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>tsuki/rupture_cleave</t>
+          <t>Tsuki/RuptureCleave</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>rupture_cleave</t>
+          <t>RuptureCleave</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>on_stance</t>
+          <t>OnStance</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1798,12 +1798,12 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>shield</t>
+          <t>Shield</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>Self</t>
         </is>
       </c>
       <c r="L22" t="n">
@@ -1816,27 +1816,27 @@
     <row r="23">
       <c r="B23" t="inlineStr">
         <is>
-          <t>tsuki_rupture_cleave_sun_add_hit</t>
+          <t>TsukiRuptureCleaveSunAddHit</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>tsuki/rupture_cleave</t>
+          <t>Tsuki/RuptureCleave</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>rupture_cleave</t>
+          <t>RuptureCleave</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>on_stance</t>
+          <t>OnStance</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1846,7 +1846,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>add_hit</t>
+          <t>AddHit</t>
         </is>
       </c>
       <c r="M23" t="n">
@@ -1859,37 +1859,37 @@
     <row r="24">
       <c r="B24" t="inlineStr">
         <is>
-          <t>tsuki_halfmoon_combo_damage_1</t>
+          <t>TsukiHalfmoonComboDamage1</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>tsuki/halfmoon_combo</t>
+          <t>Tsuki/HalfmoonCombo</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>halfmoon_combo</t>
+          <t>HalfmoonCombo</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>on_play</t>
+          <t>OnPlay</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>Damage</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>enemy</t>
+          <t>Enemy</t>
         </is>
       </c>
       <c r="L24" t="n">
@@ -1902,37 +1902,37 @@
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
-          <t>tsuki_halfmoon_combo_damage_2</t>
+          <t>TsukiHalfmoonComboDamage2</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>tsuki/halfmoon_combo</t>
+          <t>Tsuki/HalfmoonCombo</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>halfmoon_combo</t>
+          <t>HalfmoonCombo</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>on_play</t>
+          <t>OnPlay</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>Damage</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>enemy</t>
+          <t>Enemy</t>
         </is>
       </c>
       <c r="L25" t="n">
@@ -1942,37 +1942,37 @@
     <row r="26">
       <c r="B26" t="inlineStr">
         <is>
-          <t>tsuki_halfmoon_combo_damage_3</t>
+          <t>TsukiHalfmoonComboDamage3</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>tsuki/halfmoon_combo</t>
+          <t>Tsuki/HalfmoonCombo</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>halfmoon_combo</t>
+          <t>HalfmoonCombo</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>on_play</t>
+          <t>OnPlay</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>Damage</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>enemy</t>
+          <t>Enemy</t>
         </is>
       </c>
       <c r="L26" t="n">
@@ -1982,27 +1982,27 @@
     <row r="27">
       <c r="B27" t="inlineStr">
         <is>
-          <t>tsuki_halfmoon_combo_moon_add_stance</t>
+          <t>TsukiHalfmoonComboMoonAddStance</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>tsuki/halfmoon_combo</t>
+          <t>Tsuki/HalfmoonCombo</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>halfmoon_combo</t>
+          <t>HalfmoonCombo</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>on_stance</t>
+          <t>OnStance</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2012,7 +2012,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>add_card_to_hand</t>
+          <t>AddCardToHand</t>
         </is>
       </c>
       <c r="M27" t="n">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>stance_shift</t>
+          <t>StanceShift</t>
         </is>
       </c>
       <c r="Q27" t="n">
@@ -2030,27 +2030,27 @@
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
-          <t>tsuki_halfmoon_combo_sun_damage_up</t>
+          <t>TsukiHalfmoonComboSunDamageUp</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>tsuki/halfmoon_combo</t>
+          <t>Tsuki/HalfmoonCombo</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>halfmoon_combo</t>
+          <t>HalfmoonCombo</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>on_stance</t>
+          <t>OnStance</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>damage_delta</t>
+          <t>DamageDelta</t>
         </is>
       </c>
       <c r="L28" t="n">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>stance_changed_this_turn</t>
+          <t>StanceChangedThisTurn</t>
         </is>
       </c>
       <c r="Q28" t="n">
@@ -2123,27 +2123,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>character</t>
+          <t>Character</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>Id</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>display_name</t>
+          <t>DisplayName</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>Cost</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>card_type</t>
+          <t>CardType</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -2153,12 +2153,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>copies</t>
+          <t>Copies</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>keywords[]</t>
+          <t>Keywords[]</t>
         </is>
       </c>
     </row>
@@ -2249,12 +2249,12 @@
     <row r="5" ht="15" customHeight="1">
       <c r="B5" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>crescent_slash</t>
+          <t>CrescentSlash</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -2267,7 +2267,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>attack</t>
+          <t>Attack</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2289,12 +2289,12 @@
     <row r="6" ht="15" customHeight="1">
       <c r="B6" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>flow_guard</t>
+          <t>FlowGuard</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>skill</t>
+          <t>Skill</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -2329,12 +2329,12 @@
     <row r="7" ht="15" customHeight="1">
       <c r="B7" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>stance_shift</t>
+          <t>StanceShift</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2347,7 +2347,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>skill</t>
+          <t>Skill</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -2369,12 +2369,12 @@
     <row r="8" ht="26.39999961853027" customHeight="1">
       <c r="B8" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>afterimage_thrust</t>
+          <t>AfterimageThrust</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>attack</t>
+          <t>Attack</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -2409,12 +2409,12 @@
     <row r="9" ht="15" customHeight="1">
       <c r="B9" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>breath_reset</t>
+          <t>BreathReset</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>skill</t>
+          <t>Skill</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -2449,12 +2449,12 @@
     <row r="10" ht="26.39999961853027" customHeight="1">
       <c r="B10" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>rupture_cleave</t>
+          <t>RuptureCleave</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>attack</t>
+          <t>Attack</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -2489,12 +2489,12 @@
     <row r="11" ht="26.39999961853027" customHeight="1">
       <c r="B11" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>halfmoon_combo</t>
+          <t>HalfmoonCombo</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>attack</t>
+          <t>Attack</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -2569,17 +2569,17 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>keyword</t>
+          <t>Keyword</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>Description</t>
         </is>
       </c>
     </row>
@@ -3582,42 +3582,42 @@
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>#data</t>
+          <t>#archive</t>
         </is>
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>character</t>
+          <t>Character</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>Level</t>
         </is>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>attack_power</t>
+          <t>Attack</t>
         </is>
       </c>
       <c r="E2" s="10" t="inlineStr">
         <is>
-          <t>defense_power</t>
+          <t>Defense</t>
         </is>
       </c>
       <c r="F2" s="10" t="inlineStr">
         <is>
-          <t>max_hp</t>
+          <t>MaxHp</t>
         </is>
       </c>
       <c r="G2" s="10" t="inlineStr">
         <is>
-          <t>crit_rate</t>
+          <t>CritRate</t>
         </is>
       </c>
       <c r="H2" s="10" t="inlineStr">
         <is>
-          <t>crit_damage</t>
+          <t>CritDamage</t>
         </is>
       </c>
     </row>
@@ -3701,7 +3701,7 @@
       <c r="A5" s="5" t="n"/>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="C5" s="5" t="n">
@@ -3727,7 +3727,7 @@
       <c r="A6" s="5" t="n"/>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="C6" s="5" t="n">
@@ -3753,7 +3753,7 @@
       <c r="A7" s="5" t="n"/>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="C7" s="5" t="n">
@@ -3779,7 +3779,7 @@
       <c r="A8" s="5" t="n"/>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="C8" s="5" t="n">
@@ -3805,7 +3805,7 @@
       <c r="A9" s="5" t="n"/>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="C9" s="5" t="n">
@@ -3831,7 +3831,7 @@
       <c r="A10" s="5" t="n"/>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="C10" s="5" t="n">
@@ -3857,7 +3857,7 @@
       <c r="A11" s="6" t="n"/>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
@@ -3912,19 +3912,19 @@
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>Id</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>tsuki</t>
+          <t>Tsuki</t>
         </is>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>display_name</t>
+          <t>DisplayName</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -3936,7 +3936,7 @@
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>max_hp</t>
+          <t>MaxHp</t>
         </is>
       </c>
       <c r="B4" s="5" t="n">
@@ -3946,7 +3946,7 @@
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>attack_power</t>
+          <t>Attack</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
@@ -3956,7 +3956,7 @@
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>defense_power</t>
+          <t>Defense</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
@@ -3966,7 +3966,7 @@
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>starting_energy</t>
+          <t>StartingEnergy</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
@@ -3976,7 +3976,7 @@
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>crit_rate</t>
+          <t>CritRate</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
@@ -3986,7 +3986,7 @@
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>crit_damage</t>
+          <t>CritDamage</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
@@ -4001,7 +4001,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>data/player/PlayerStats.tres</t>
+          <t>data/Player/PlayerStats.tres</t>
         </is>
       </c>
     </row>
@@ -4057,37 +4057,37 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>Id</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>display_name</t>
+          <t>DisplayName</t>
         </is>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>max_hp</t>
+          <t>MaxHp</t>
         </is>
       </c>
       <c r="E2" s="10" t="inlineStr">
         <is>
-          <t>attack_power</t>
+          <t>Attack</t>
         </is>
       </c>
       <c r="F2" s="10" t="inlineStr">
         <is>
-          <t>defense_power</t>
+          <t>Defense</t>
         </is>
       </c>
       <c r="G2" s="10" t="inlineStr">
         <is>
-          <t>crit_rate</t>
+          <t>CritRate</t>
         </is>
       </c>
       <c r="H2" s="10" t="inlineStr">
         <is>
-          <t>crit_damage</t>
+          <t>CritDamage</t>
         </is>
       </c>
       <c r="I2" s="10" t="inlineStr">
@@ -4186,7 +4186,7 @@
       <c r="A5" s="5" t="n"/>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>abyssal_crown_guardian</t>
+          <t>AbyssalCrownGuardian</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -4219,7 +4219,7 @@
       <c r="A6" s="5" t="n"/>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>bog_stalker</t>
+          <t>BogStalker</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -4252,7 +4252,7 @@
       <c r="A7" s="5" t="n"/>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>bone_crawler</t>
+          <t>BoneCrawler</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -4285,7 +4285,7 @@
       <c r="A8" s="5" t="n"/>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>crown_acolyte</t>
+          <t>CrownAcolyte</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -4318,7 +4318,7 @@
       <c r="A9" s="5" t="n"/>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>frost_revenant</t>
+          <t>FrostRevenant</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -4351,7 +4351,7 @@
       <c r="A10" s="5" t="n"/>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>gravebound_crawler</t>
+          <t>GraveboundCrawler</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -4384,7 +4384,7 @@
       <c r="A11" s="5" t="n"/>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>mire_imp</t>
+          <t>MireImp</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -4417,7 +4417,7 @@
       <c r="A12" s="6" t="n"/>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>monster_dummy</t>
+          <t>MonsterDummy</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -4500,42 +4500,42 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>Id</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>display_name</t>
+          <t>DisplayName</t>
         </is>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>stats_path</t>
+          <t>StatsPath</t>
         </is>
       </c>
       <c r="E2" s="10" t="inlineStr">
         <is>
-          <t>scene_path</t>
+          <t>ScenePath</t>
         </is>
       </c>
       <c r="F2" s="10" t="inlineStr">
         <is>
-          <t>intent_sequence</t>
+          <t>IntentSequence</t>
         </is>
       </c>
       <c r="G2" s="10" t="inlineStr">
         <is>
-          <t>action_count</t>
+          <t>ActionCount</t>
         </is>
       </c>
       <c r="H2" s="10" t="inlineStr">
         <is>
-          <t>hp_bar_offset</t>
+          <t>HpBarOffset</t>
         </is>
       </c>
       <c r="I2" s="10" t="inlineStr">
         <is>
-          <t>intent_overlay_offset</t>
+          <t>IntentOverlayOffset</t>
         </is>
       </c>
       <c r="J2" s="10" t="inlineStr">
@@ -4644,7 +4644,7 @@
       <c r="A5" s="5" t="n"/>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>abyssal_crown_guardian</t>
+          <t>AbyssalCrownGuardian</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -4659,7 +4659,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>res://scenes/monster/monster_abyssal_crown_guardian.tscn</t>
+          <t>res://scenes/monster/MonsterAbyssalCrownGuardian.tscn</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
@@ -4690,7 +4690,7 @@
       <c r="A6" s="5" t="n"/>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>bog_stalker</t>
+          <t>BogStalker</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -4705,7 +4705,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>res://scenes/monster/monster_bog_stalker.tscn</t>
+          <t>res://scenes/monster/MonsterBogStalker.tscn</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -4736,7 +4736,7 @@
       <c r="A7" s="5" t="n"/>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>bone_crawler</t>
+          <t>BoneCrawler</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -4751,7 +4751,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>res://scenes/monster/monster_bone_crawler.tscn</t>
+          <t>res://scenes/monster/MonsterBoneCrawler.tscn</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
@@ -4782,7 +4782,7 @@
       <c r="A8" s="5" t="n"/>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>crown_acolyte</t>
+          <t>CrownAcolyte</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>res://scenes/monster/monster_crown_acolyte.tscn</t>
+          <t>res://scenes/monster/MonsterCrownAcolyte.tscn</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -4828,7 +4828,7 @@
       <c r="A9" s="5" t="n"/>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>frost_revenant</t>
+          <t>FrostRevenant</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -4843,7 +4843,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>res://scenes/monster/monster_frost_revenant.tscn</t>
+          <t>res://scenes/monster/MonsterFrostRevenant.tscn</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -4874,7 +4874,7 @@
       <c r="A10" s="5" t="n"/>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>gravebound_crawler</t>
+          <t>GraveboundCrawler</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -4889,7 +4889,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>res://scenes/monster/monster_gravebound_crawler.tscn</t>
+          <t>res://scenes/monster/MonsterGraveboundCrawler.tscn</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -4920,7 +4920,7 @@
       <c r="A11" s="6" t="n"/>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>mire_imp</t>
+          <t>MireImp</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -4935,7 +4935,7 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>res://scenes/monster/monster_mire_imp.tscn</t>
+          <t>res://scenes/monster/MonsterMireImp.tscn</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -5012,32 +5012,32 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>Id</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>display_name</t>
+          <t>DisplayName</t>
         </is>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>intent_type</t>
+          <t>IntentType</t>
         </is>
       </c>
       <c r="E2" s="10" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>Amount</t>
         </is>
       </c>
       <c r="F2" s="10" t="inlineStr">
         <is>
-          <t>icon_label</t>
+          <t>IconLabel</t>
         </is>
       </c>
       <c r="G2" s="10" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="H2" s="10" t="inlineStr">
@@ -5296,7 +5296,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>player_growth and monster_stats exporter-compatible sheets.</t>
+          <t>PlayerGrowth and MonsterStats exporter-compatible sheets.</t>
         </is>
       </c>
     </row>

</xml_diff>